<commit_message>
Pruebas de lora completas
</commit_message>
<xml_diff>
--- a/CUADRO DE PRUEBAS.xlsx
+++ b/CUADRO DE PRUEBAS.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\omich\Documents\SolucionesEnergeticasParaWSN\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C265AFA3-8303-42AF-86A3-85E7F6F6699E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{57A5C65B-D0A7-4438-8C94-50EB2D8767BE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{16E32420-E92C-48F4-9AFE-AC6FE85723F6}"/>
   </bookViews>
@@ -40,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="179" uniqueCount="57">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="183" uniqueCount="59">
   <si>
     <t>XBEE</t>
   </si>
@@ -211,6 +211,12 @@
   </si>
   <si>
     <t>ENERGY + ADAPTIVE</t>
+  </si>
+  <si>
+    <t>71.7 ms</t>
+  </si>
+  <si>
+    <t>61.9 mAh</t>
   </si>
 </sst>
 </file>
@@ -834,10 +840,18 @@
       <c r="E8" s="2" t="s">
         <v>13</v>
       </c>
-      <c r="F8" s="2"/>
-      <c r="G8" s="2"/>
-      <c r="H8" s="2"/>
-      <c r="I8" s="2"/>
+      <c r="F8" s="2" t="s">
+        <v>54</v>
+      </c>
+      <c r="G8" s="2" t="s">
+        <v>58</v>
+      </c>
+      <c r="H8" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="I8" s="2" t="s">
+        <v>57</v>
+      </c>
     </row>
     <row r="9" spans="2:9" x14ac:dyDescent="0.3">
       <c r="B9" s="2">

</xml_diff>